<commit_message>
Refactor and extend economic multifunctionality plotting
Rewrote and expanded the ggplot code for economic multifunctionality vs sown plant diversity, adding support for multiple price scenarios, improved axis scaling, and enhanced legend and theme customization. Also added data preparation steps for plotting and saving the output figure, improving clarity and flexibility for visualizing scenario comparisons.
</commit_message>
<xml_diff>
--- a/Data Analysis/1_Data/C&N_Soil/179_5_data.xlsx
+++ b/Data Analysis/1_Data/C&N_Soil/179_5_data.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" hidePivotFieldList="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA40DEC-6E14-45A8-9A60-1FFC61D06527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25C04933-680A-49EE-8DA0-FCD5CA4A43FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId2"/>
+    <pivotCache cacheId="0" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="750" uniqueCount="112">
   <si>
     <t>plot</t>
   </si>
@@ -7065,7 +7065,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BAFF5916-46E8-4082-855F-F71D4DCAC4F5}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BAFF5916-46E8-4082-855F-F71D4DCAC4F5}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="L1:M101" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0">
@@ -8218,7 +8218,10 @@
         <v>1.3399999999999999</v>
       </c>
       <c r="P11" s="8"/>
-      <c r="Q11" s="9"/>
+      <c r="Q11" s="9">
+        <f>AVERAGE(Q14,P28)</f>
+        <v>1.3033333333333332</v>
+      </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
@@ -8881,7 +8884,9 @@
       <c r="M28" s="7">
         <v>1.3049999999999999</v>
       </c>
-      <c r="P28" s="8"/>
+      <c r="P28" s="8">
+        <v>1.3049999999999999</v>
+      </c>
       <c r="Q28" s="9"/>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
@@ -9197,7 +9202,8 @@
         <v>1.2650000000000001</v>
       </c>
       <c r="R37">
-        <v>1.2650000000000001</v>
+        <f>AVERAGE(Q37,Q49)</f>
+        <v>1.2975000000000001</v>
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.25">
@@ -9241,7 +9247,8 @@
         <v>1.2750000000000001</v>
       </c>
       <c r="R38">
-        <v>1.2750000000000001</v>
+        <f>AVERAGE(Q38,Q50)</f>
+        <v>1.3</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
@@ -9282,7 +9289,8 @@
         <v>1.2416666666666669</v>
       </c>
       <c r="R39">
-        <v>1.2416666666666669</v>
+        <f>AVERAGE(Q39,Q51)</f>
+        <v>1.2791666666666668</v>
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
@@ -9323,7 +9331,8 @@
         <v>1.2716666666666667</v>
       </c>
       <c r="R40">
-        <v>1.2716666666666667</v>
+        <f t="shared" ref="R38:R47" si="0">AVERAGE(Q40,Q52)</f>
+        <v>1.2666666666666666</v>
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.25">
@@ -9364,7 +9373,8 @@
         <v>1.2283333333333333</v>
       </c>
       <c r="R41">
-        <v>1.2283333333333333</v>
+        <f t="shared" si="0"/>
+        <v>1.2424999999999999</v>
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
@@ -9405,7 +9415,8 @@
         <v>1.2416666666666667</v>
       </c>
       <c r="R42">
-        <v>1.2416666666666667</v>
+        <f t="shared" si="0"/>
+        <v>1.2616666666666667</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.25">
@@ -9446,7 +9457,8 @@
         <v>1.1983333333333333</v>
       </c>
       <c r="R43">
-        <v>1.1983333333333333</v>
+        <f t="shared" si="0"/>
+        <v>1.2291666666666665</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
@@ -9490,7 +9502,8 @@
         <v>1.26</v>
       </c>
       <c r="R44">
-        <v>1.26</v>
+        <f t="shared" si="0"/>
+        <v>1.2633333333333332</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
@@ -9531,7 +9544,8 @@
         <v>1.2266666666666668</v>
       </c>
       <c r="R45">
-        <v>1.2266666666666668</v>
+        <f t="shared" si="0"/>
+        <v>1.2308333333333334</v>
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.25">
@@ -9572,7 +9586,8 @@
         <v>1.1983333333333333</v>
       </c>
       <c r="R46">
-        <v>1.1983333333333333</v>
+        <f t="shared" si="0"/>
+        <v>1.2033333333333331</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
@@ -9613,7 +9628,8 @@
         <v>1.165</v>
       </c>
       <c r="R47">
-        <v>1.165</v>
+        <f t="shared" si="0"/>
+        <v>1.1816666666666666</v>
       </c>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.25">
@@ -9681,8 +9697,12 @@
       <c r="M49" s="7">
         <v>1.3516666666666666</v>
       </c>
-      <c r="P49" s="8"/>
-      <c r="Q49" s="9"/>
+      <c r="P49" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q49" s="9">
+        <v>1.33</v>
+      </c>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
@@ -9718,8 +9738,12 @@
       <c r="M50" s="7">
         <v>1.3233333333333333</v>
       </c>
-      <c r="P50" s="8"/>
-      <c r="Q50" s="9"/>
+      <c r="P50" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q50" s="9">
+        <v>1.325</v>
+      </c>
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
@@ -9752,8 +9776,12 @@
       <c r="M51" s="7">
         <v>1.2949999999999999</v>
       </c>
-      <c r="P51" s="8"/>
-      <c r="Q51" s="9"/>
+      <c r="P51" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q51" s="9">
+        <v>1.3166666666666667</v>
+      </c>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
@@ -9786,8 +9814,12 @@
       <c r="M52" s="7">
         <v>1.33</v>
       </c>
-      <c r="P52" s="8"/>
-      <c r="Q52" s="9"/>
+      <c r="P52" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q52" s="9">
+        <v>1.2616666666666667</v>
+      </c>
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
@@ -9820,8 +9852,12 @@
       <c r="M53" s="7">
         <v>1.325</v>
       </c>
-      <c r="P53" s="8"/>
-      <c r="Q53" s="9"/>
+      <c r="P53" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q53" s="9">
+        <v>1.2566666666666666</v>
+      </c>
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
@@ -9854,8 +9890,12 @@
       <c r="M54" s="7">
         <v>1.3166666666666667</v>
       </c>
-      <c r="P54" s="8"/>
-      <c r="Q54" s="9"/>
+      <c r="P54" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q54" s="9">
+        <v>1.2816666666666665</v>
+      </c>
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
@@ -9888,8 +9928,12 @@
       <c r="M55" s="7">
         <v>1.2616666666666667</v>
       </c>
-      <c r="P55" s="8"/>
-      <c r="Q55" s="9"/>
+      <c r="P55" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q55" s="9">
+        <v>1.26</v>
+      </c>
     </row>
     <row r="56" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
@@ -9925,8 +9969,12 @@
       <c r="M56" s="7">
         <v>1.2566666666666666</v>
       </c>
-      <c r="P56" s="8"/>
-      <c r="Q56" s="9"/>
+      <c r="P56" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q56" s="9">
+        <v>1.2666666666666666</v>
+      </c>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
@@ -9959,8 +10007,12 @@
       <c r="M57" s="7">
         <v>1.2816666666666665</v>
       </c>
-      <c r="P57" s="8"/>
-      <c r="Q57" s="9"/>
+      <c r="P57" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q57" s="9">
+        <v>1.2350000000000001</v>
+      </c>
     </row>
     <row r="58" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
@@ -9993,8 +10045,12 @@
       <c r="M58" s="7">
         <v>1.26</v>
       </c>
-      <c r="P58" s="8"/>
-      <c r="Q58" s="9"/>
+      <c r="P58" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q58" s="9">
+        <v>1.2083333333333333</v>
+      </c>
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
@@ -10027,8 +10083,12 @@
       <c r="M59" s="7">
         <v>1.2666666666666666</v>
       </c>
-      <c r="P59" s="8"/>
-      <c r="Q59" s="9"/>
+      <c r="P59" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q59" s="9">
+        <v>1.1983333333333333</v>
+      </c>
     </row>
     <row r="60" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">

</xml_diff>